<commit_message>
removing availabilty from books and moving to bookcopy, adding books in bulk works if formatted correctly
</commit_message>
<xml_diff>
--- a/bib-backend/src/main/resources/templates/books_template.xlsx
+++ b/bib-backend/src/main/resources/templates/books_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apbe-my.sharepoint.com/personal/s140265_ap_be/Documents/j4 semester 2/software project/gosmartlib/bib-backend/src/main/resources/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="8_{27C54EC1-E7C2-4326-A747-34623A4C1D1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0C4A4F20-1B81-4A53-81C0-A2647274A30B}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="8_{27C54EC1-E7C2-4326-A747-34623A4C1D1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F1F9ADD4-5320-4628-8F4B-F3DED6CBD004}"/>
   <bookViews>
-    <workbookView xWindow="1950" yWindow="1080" windowWidth="21960" windowHeight="11265" xr2:uid="{966E3E03-C773-47F2-B79B-3CCE2F09ED19}"/>
+    <workbookView xWindow="2970" yWindow="5370" windowWidth="22770" windowHeight="11235" xr2:uid="{966E3E03-C773-47F2-B79B-3CCE2F09ED19}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>ISBN</t>
   </si>
@@ -57,12 +57,6 @@
   </si>
   <si>
     <t>releaseYear</t>
-  </si>
-  <si>
-    <t>availability</t>
-  </si>
-  <si>
-    <t>AVAILABLE</t>
   </si>
 </sst>
 </file>
@@ -115,6 +109,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -434,7 +432,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEFECC34-77A1-46E4-A3E3-F6F11B9BA77B}">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.140625" bestFit="1" customWidth="1"/>
@@ -446,7 +444,7 @@
     <col min="8" max="8" width="10.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -467,14 +465,6 @@
       </c>
       <c r="G1" t="s">
         <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="H2" t="s">
-        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
adding reading level to books
</commit_message>
<xml_diff>
--- a/bib-backend/src/main/resources/templates/books_template.xlsx
+++ b/bib-backend/src/main/resources/templates/books_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apbe-my.sharepoint.com/personal/s140265_ap_be/Documents/j4 semester 2/software project/gosmartlib/bib-backend/src/main/resources/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="8_{27C54EC1-E7C2-4326-A747-34623A4C1D1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F1F9ADD4-5320-4628-8F4B-F3DED6CBD004}"/>
+  <xr:revisionPtr revIDLastSave="34" documentId="8_{27C54EC1-E7C2-4326-A747-34623A4C1D1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4ACD3A7A-A7CA-4489-84CD-E91461BDDD57}"/>
   <bookViews>
-    <workbookView xWindow="2970" yWindow="5370" windowWidth="22770" windowHeight="11235" xr2:uid="{966E3E03-C773-47F2-B79B-3CCE2F09ED19}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{966E3E03-C773-47F2-B79B-3CCE2F09ED19}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="11">
   <si>
     <t>ISBN</t>
   </si>
@@ -57,16 +57,34 @@
   </si>
   <si>
     <t>releaseYear</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Genre 1 </t>
+  </si>
+  <si>
+    <t>Genre 2</t>
+  </si>
+  <si>
+    <t>Genre 3</t>
+  </si>
+  <si>
+    <t>Graphic novel / strip</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -432,7 +450,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DEFECC34-77A1-46E4-A3E3-F6F11B9BA77B}">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.140625" bestFit="1" customWidth="1"/>
@@ -441,10 +459,12 @@
     <col min="4" max="4" width="6.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.85546875" customWidth="1"/>
+    <col min="9" max="9" width="18.5703125" customWidth="1"/>
+    <col min="10" max="10" width="18.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -466,11 +486,32 @@
       <c r="G1" t="s">
         <v>6</v>
       </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="H2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I2" t="s">
+        <v>10</v>
+      </c>
+      <c r="J2" t="s">
+        <v>10</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2" xr:uid="{A77FFDC8-26BB-4678-A8F6-62AEB7F5D98D}">
-      <formula1>"AVAILABLE,BORROWED,DAMAGED,LOST"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:J2" xr:uid="{4895184D-3A4C-4850-A54C-713B6A841E62}">
+      <formula1>"Fictie algemeen,Literaire roman,Spanning / thriller,Detective / misdaad,Fantasy,Sciencefiction,Dystopie,Historische roman,Romantiek,Coming-of-age,Avontuur,Oorlog &amp; conflict,Horror,Humor,Graphic novel / strip,Poëzie,Non-fictie algemeen"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>